<commit_message>
Preserve source workbook style with readable complete headers
</commit_message>
<xml_diff>
--- a/outputs/Figure_1.xlsx
+++ b/outputs/Figure_1.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contents" sheetId="1" r:id="Rf53346b923f34d30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig1_region_values" sheetId="2" r:id="R927475d3af1b44a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig1_quartile_statistics" sheetId="3" r:id="R694b1cb6e8dc4d1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig1_baseline_change_summary" sheetId="4" r:id="Ra089a368db1f44fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig1_association" sheetId="5" r:id="R9c3eba2d45f34c9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contents" sheetId="1" r:id="R8789315e17b74968"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig1_region_values" sheetId="2" r:id="Rdef5a14a54ed4126"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig1_quartile_statistics" sheetId="3" r:id="Rf9139517178f489e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig1_baseline_change_summary" sheetId="4" r:id="Rb69f77e2804742fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig1_association" sheetId="5" r:id="R50e60dde4d8c4dc4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -283,7 +283,7 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="16.8799991607666" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="36" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="48" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="16.8799991607666" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="80" hidden="0" customWidth="1"/>
   </x:cols>

</xml_diff>